<commit_message>
PAUSED (task144): architecture 2 built and gated, stage 4 round 2 running
The portal's FAILED_TO_STUMP (both responses landed slidewell at 12,000 with
9,000 added) is answered by architecture 2: the field notes and manifest are
gone, every file carries its own conventions, the twin pair is removed, and the
decisive step is the period the follower-view rate is read over (from day 8,
after a forum-carried launch week), which files kilnkit at about 12,000 with
9,000 added. Stage 4 round 1: both scored readers missed the call (tracewire)
and took every ask figure, so the asks were re-sited onto mail gateways' link
fetches and a member merging accounts on leaving, and the prompt asks for those
figures. Resume: score readers C and D and finish the re-judge on f0ae1a2f.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Jt4Mt622iBfGoK24ivCU
</commit_message>
<xml_diff>
--- a/task144/golden/sluis_spotlight_2026-10.xlsx
+++ b/task144/golden/sluis_spotlight_2026-10.xlsx
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="83">
-  <si>
-    <t>October 2026 Sluis spotlight: slidewell, about 12,000 external stars expected in its first 90 days public</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="85">
+  <si>
+    <t>October 2026 Sluis spotlight: kilnkit, about 12,000 external stars expected in its first 90 days public</t>
   </si>
   <si>
     <t>Pick under the featuring memo of 15 September 2026 for the issue of Tuesday 6 October 2026, from the warehouse extract to 27 September 2026. Expected stars to the nearest thousand.</t>
@@ -33,7 +33,7 @@
     <t>Spotlight</t>
   </si>
   <si>
-    <t>slidewell (pjvdlinden/slidewell)</t>
+    <t>kilnkit (kilnworks/kilnkit)</t>
   </si>
   <si>
     <t>Expected external stars in its first 90 days public, if spotlighted</t>
@@ -42,7 +42,7 @@
     <t>Of which the spotlight adds</t>
   </si>
   <si>
-    <t>Next: tracewire, at 9,000</t>
+    <t>Next: slidewell and tracewire, each at about 10,000</t>
   </si>
   <si>
     <t>Repository</t>
@@ -63,13 +63,16 @@
     <t>Expected without the spotlight, day 90</t>
   </si>
   <si>
-    <t>Feed-card stars to 27 Sep</t>
-  </si>
-  <si>
-    <t>Followers of its starrers</t>
-  </si>
-  <si>
-    <t>Stars per follower view (%)</t>
+    <t>Stars per follower view over its life (%)</t>
+  </si>
+  <si>
+    <t>Feed-card stars from day 8</t>
+  </si>
+  <si>
+    <t>Followers of its starrers from day 8</t>
+  </si>
+  <si>
+    <t>Stars per follower view from day 8 (%)</t>
   </si>
   <si>
     <t>Stars the spotlight adds</t>
@@ -78,6 +81,15 @@
     <t>Expected external stars, first 90 days, if spotlighted</t>
   </si>
   <si>
+    <t>kilnkit</t>
+  </si>
+  <si>
+    <t>kilnworks</t>
+  </si>
+  <si>
+    <t>29 Aug 2026 13:25</t>
+  </si>
+  <si>
     <t>slidewell</t>
   </si>
   <si>
@@ -96,6 +108,15 @@
     <t>26 Aug 2026 09:14</t>
   </si>
   <si>
+    <t>shiftgres</t>
+  </si>
+  <si>
+    <t>lindengracht-dev</t>
+  </si>
+  <si>
+    <t>03 Sep 2026 07:02</t>
+  </si>
+  <si>
     <t>ferrolog</t>
   </si>
   <si>
@@ -105,24 +126,6 @@
     <t>07 Sep 2026 08:37</t>
   </si>
   <si>
-    <t>shiftgres</t>
-  </si>
-  <si>
-    <t>lindengracht-dev</t>
-  </si>
-  <si>
-    <t>03 Sep 2026 07:02</t>
-  </si>
-  <si>
-    <t>kilnkit</t>
-  </si>
-  <si>
-    <t>kilnworks</t>
-  </si>
-  <si>
-    <t>29 Aug 2026 13:25</t>
-  </si>
-  <si>
     <t>hullcheck</t>
   </si>
   <si>
@@ -162,13 +165,16 @@
     <t>Without the spotlight: external stars to 27 September plus the last seven days' daily pace times the ratio of stars still to come by day 90 to that pace, at the same age, among the lottery's runners-up.</t>
   </si>
   <si>
-    <t>The spotlight adds the issue's own newsletter stars and the stars they set off: each star shows in the starrer's followers' home feeds, where followers star at the repository's own rate per follower view (feed-card stars over the followers of everyone who starred it), and those stars show to their followers in turn. Added stars = newsletter stars x (1 + rate x newsletter starrers' mean followers / (1 - rate x feed starrers' mean followers)).</t>
+    <t>The spotlight adds the issue's own newsletter stars and the stars they set off: each star shows in the starrer's followers' home feeds, where followers star at the repository's rate per follower view, and those stars show to their followers in turn. Added stars = newsletter stars x (1 + rate x newsletter starrers' mean followers / (1 - rate x feed starrers' mean followers)).</t>
+  </si>
+  <si>
+    <t>The rate per view is read from day 8 public on (feed-card stars over the followers of everyone who starred it from that day): while a repository is on an outside forum's front page, followers who see it starred have often seen it there already and star from the card more readily, and the October readers' stars will come weeks after any launch. slidewell's cards converted at 1.98 per cent a view over its life and at 0.74 per cent from day 8. On the lottery's closed spotlights the day-8 rate reproduces the stars each spotlight added to within a few hundred, where the whole-life rate misses by more than a thousand.</t>
   </si>
   <si>
     <t>Sluis issues, April to September 2026: delivery and spotlight click-through</t>
   </si>
   <si>
-    <t>Delivered: subscribers the issue was delivered to (a send to a segment of the list reaches subscribers already counted). Click-through: subscribers who clicked any link to the issue's spotlighted repository, in any of the issue's sends.</t>
+    <t>Delivered: subscribers the issue was delivered to (the Thursday send to non-openers reaches subscribers already counted). Clicked through: subscribers who clicked a link to the issue's spotlighted repository themselves, in any of the issue's sends; a mail gateway's check of every link of a message on delivery is not a click.</t>
   </si>
   <si>
     <t>Issue</t>
@@ -234,7 +240,7 @@
     <t>October 2026 shortlist: who nominated each repository</t>
   </si>
   <si>
-    <t>People, not form responses: a signed-out response is matched to the account whose primary email it is, a merged account to the account it was merged into, and a renamed repository's old name to the repository. Outside: not a member of the owning organisation when nominating.</t>
+    <t>People, not form responses: a signed-out response is matched to the account whose primary email it is, a merged account to the account it was merged into, and a renamed repository's old name to the repository. Outside: not a member of the owning organisation when nominating, through any of their accounts, those later merged into the one they nominated from included.</t>
   </si>
   <si>
     <t>People who nominated it</t>
@@ -267,20 +273,19 @@
     <t>Spotlight sheet: expected stars, stars without the spotlight and stars the spotlight adds are rounded to the nearest thousand from unrounded figures; stars to 27 September, feed-card stars and followers are counts.</t>
   </si>
   <si>
-    <t>Sluis issues: Postwerk to the May issue, Relaymark from June. Each issue went to the Sluis list in two batches on its Tuesday and again on the Thursday to subscribers who had not opened it; delivered counts the Tuesday batches, click-through counts subscribers clicking the spotlight's heading, screenshot or button in any of the three sends. Test sends to the editorial seed addresses and Product News are left out.</t>
-  </si>
-  <si>
-    <t>Nominations: responses to the October form. A signed-out response is matched to the account whose primary email it is, a merged account to the account it was merged into, kiln-ui to kilnkit and imagelint to hullcheck; addresses of forks under other owners are not nominations of the shortlisted repository.</t>
+    <t>Sluis issues: Postwerk to the May issue, Relaymark from June. Each issue went to the Sluis list in two batches on its Tuesday and again on the Thursday to subscribers who had not opened it; delivered counts the Tuesday batches, click-through counts subscribers clicking the spotlight's heading, screenshot or button in any of the three sends. Some subscribers' mail gateways open every link of a message the second it is delivered: Relaymark logs that as four or more links clicked within two seconds, Postwerk as one click on every link of the send, and those fetches are left out (the platforms' own click counts leave out only the gateways they recognise). Test sends to the editorial seed addresses and Product News are left out.</t>
+  </si>
+  <si>
+    <t>Nominations: responses to the October form. A signed-out response is matched to the account whose primary email it is, a merged account to the account it was merged into, kiln-ui to kilnkit and imagelint to hullcheck; addresses of forks under other owners are not nominations of the shortlisted repository. Five nominators used a personal account while still members through a work account that they merged into it when they left, a few days later: they nominated from inside.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -370,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -387,14 +392,15 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -713,7 +719,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -723,23 +729,24 @@
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="6" width="14.7109375" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -747,7 +754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
@@ -755,7 +762,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -763,12 +770,12 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="46" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -802,311 +809,341 @@
       <c r="K9" s="7" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10" s="10">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E10" s="11">
-        <v>2766</v>
+        <v>1523</v>
       </c>
       <c r="F10" s="11">
         <v>3000</v>
       </c>
-      <c r="G10" s="11">
-        <v>551</v>
+      <c r="G10" s="12">
+        <v>1.79</v>
       </c>
       <c r="H10" s="11">
-        <v>30671</v>
-      </c>
-      <c r="I10" s="12">
-        <v>1.796</v>
-      </c>
-      <c r="J10" s="11">
+        <v>356</v>
+      </c>
+      <c r="I10" s="11">
+        <v>19548</v>
+      </c>
+      <c r="J10" s="13">
+        <v>1.82</v>
+      </c>
+      <c r="K10" s="11">
         <v>9000</v>
       </c>
-      <c r="K10" s="13">
+      <c r="L10" s="14">
         <v>12000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="15">
+        <v>35</v>
+      </c>
+      <c r="E11" s="16">
+        <v>4175</v>
+      </c>
+      <c r="F11" s="16">
+        <v>5000</v>
+      </c>
+      <c r="G11" s="17">
+        <v>1.98</v>
+      </c>
+      <c r="H11" s="16">
+        <v>89</v>
+      </c>
+      <c r="I11" s="16">
+        <v>11949</v>
+      </c>
+      <c r="J11" s="18">
+        <v>0.74</v>
+      </c>
+      <c r="K11" s="16">
+        <v>5000</v>
+      </c>
+      <c r="L11" s="5">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="15">
+        <v>33</v>
+      </c>
+      <c r="E12" s="16">
+        <v>4534</v>
+      </c>
+      <c r="F12" s="16">
+        <v>7000</v>
+      </c>
+      <c r="G12" s="17">
+        <v>0.22</v>
+      </c>
+      <c r="H12" s="16">
+        <v>214</v>
+      </c>
+      <c r="I12" s="16">
+        <v>182308</v>
+      </c>
+      <c r="J12" s="18">
+        <v>0.12</v>
+      </c>
+      <c r="K12" s="16">
+        <v>3000</v>
+      </c>
+      <c r="L12" s="5">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="15">
+        <v>25</v>
+      </c>
+      <c r="E13" s="16">
+        <v>1630</v>
+      </c>
+      <c r="F13" s="16">
+        <v>4000</v>
+      </c>
+      <c r="G13" s="17">
+        <v>0.48</v>
+      </c>
+      <c r="H13" s="16">
+        <v>103</v>
+      </c>
+      <c r="I13" s="16">
+        <v>21033</v>
+      </c>
+      <c r="J13" s="18">
+        <v>0.49</v>
+      </c>
+      <c r="K13" s="16">
+        <v>4000</v>
+      </c>
+      <c r="L13" s="5">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="15">
         <v>21</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="E14" s="16">
+        <v>1929</v>
+      </c>
+      <c r="F14" s="16">
+        <v>4000</v>
+      </c>
+      <c r="G14" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="H14" s="16">
+        <v>92</v>
+      </c>
+      <c r="I14" s="16">
+        <v>18540</v>
+      </c>
+      <c r="J14" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="K14" s="16">
+        <v>4000</v>
+      </c>
+      <c r="L14" s="5">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="15">
         <v>23</v>
       </c>
-      <c r="D11" s="14">
-        <v>33</v>
-      </c>
-      <c r="E11" s="15">
-        <v>3876</v>
-      </c>
-      <c r="F11" s="15">
+      <c r="E15" s="16">
+        <v>1936</v>
+      </c>
+      <c r="F15" s="16">
+        <v>3000</v>
+      </c>
+      <c r="G15" s="17">
+        <v>0.4</v>
+      </c>
+      <c r="H15" s="16">
+        <v>58</v>
+      </c>
+      <c r="I15" s="16">
+        <v>23196</v>
+      </c>
+      <c r="J15" s="18">
+        <v>0.25</v>
+      </c>
+      <c r="K15" s="16">
+        <v>4000</v>
+      </c>
+      <c r="L15" s="5">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="15">
+        <v>27</v>
+      </c>
+      <c r="E16" s="16">
+        <v>1396</v>
+      </c>
+      <c r="F16" s="16">
+        <v>2000</v>
+      </c>
+      <c r="G16" s="17">
+        <v>0.32</v>
+      </c>
+      <c r="H16" s="16">
+        <v>9</v>
+      </c>
+      <c r="I16" s="16">
+        <v>5050</v>
+      </c>
+      <c r="J16" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="K16" s="16">
+        <v>4000</v>
+      </c>
+      <c r="L16" s="5">
         <v>6000</v>
       </c>
-      <c r="G11" s="15">
-        <v>446</v>
-      </c>
-      <c r="H11" s="15">
-        <v>450226</v>
-      </c>
-      <c r="I11" s="16">
-        <v>0.099</v>
-      </c>
-      <c r="J11" s="15">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J19" s="19">
+        <v>0.7111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J20" s="16">
+        <v>433812</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J21" s="16">
         <v>3000</v>
       </c>
-      <c r="K11" s="5">
-        <v>9000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="14">
-        <v>21</v>
-      </c>
-      <c r="E12" s="15">
-        <v>1892</v>
-      </c>
-      <c r="F12" s="15">
-        <v>4000</v>
-      </c>
-      <c r="G12" s="15">
-        <v>191</v>
-      </c>
-      <c r="H12" s="15">
-        <v>40549</v>
-      </c>
-      <c r="I12" s="16">
-        <v>0.471</v>
-      </c>
-      <c r="J12" s="15">
-        <v>4000</v>
-      </c>
-      <c r="K12" s="5">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="14">
-        <v>25</v>
-      </c>
-      <c r="E13" s="15">
-        <v>1826</v>
-      </c>
-      <c r="F13" s="15">
-        <v>4000</v>
-      </c>
-      <c r="G13" s="15">
-        <v>140</v>
-      </c>
-      <c r="H13" s="15">
-        <v>39636</v>
-      </c>
-      <c r="I13" s="16">
-        <v>0.353</v>
-      </c>
-      <c r="J13" s="15">
-        <v>4000</v>
-      </c>
-      <c r="K13" s="5">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="14">
-        <v>30</v>
-      </c>
-      <c r="E14" s="15">
-        <v>1245</v>
-      </c>
-      <c r="F14" s="15">
-        <v>2000</v>
-      </c>
-      <c r="G14" s="15">
-        <v>485</v>
-      </c>
-      <c r="H14" s="15">
-        <v>75098</v>
-      </c>
-      <c r="I14" s="16">
-        <v>0.646</v>
-      </c>
-      <c r="J14" s="15">
-        <v>5000</v>
-      </c>
-      <c r="K14" s="5">
-        <v>7000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="14">
-        <v>23</v>
-      </c>
-      <c r="E15" s="15">
-        <v>1912</v>
-      </c>
-      <c r="F15" s="15">
-        <v>3000</v>
-      </c>
-      <c r="G15" s="15">
-        <v>166</v>
-      </c>
-      <c r="H15" s="15">
-        <v>58747</v>
-      </c>
-      <c r="I15" s="16">
-        <v>0.283</v>
-      </c>
-      <c r="J15" s="15">
-        <v>4000</v>
-      </c>
-      <c r="K15" s="5">
-        <v>7000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="14">
-        <v>27</v>
-      </c>
-      <c r="E16" s="15">
-        <v>1299</v>
-      </c>
-      <c r="F16" s="15">
-        <v>2000</v>
-      </c>
-      <c r="G16" s="15">
-        <v>16</v>
-      </c>
-      <c r="H16" s="15">
-        <v>6586</v>
-      </c>
-      <c r="I16" s="16">
-        <v>0.243</v>
-      </c>
-      <c r="J16" s="15">
-        <v>4000</v>
-      </c>
-      <c r="K16" s="5">
-        <v>6000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I19" s="17">
-        <v>0.7236</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I20" s="15">
-        <v>433812</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I21" s="15">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="I22" s="18">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="J22" s="20">
+        <v>84.90000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="I23" s="19">
-        <v>10.27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="20" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="20" t="s">
+      <c r="J23" s="18">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
         <v>46</v>
       </c>
     </row>
+    <row r="26" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="21" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A26:K26"/>
+  <mergeCells count="3">
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A27:L27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
@@ -1127,152 +1164,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>47</v>
+      <c r="A1" s="22" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="15">
+        <v>59</v>
+      </c>
+      <c r="D5" s="16">
         <v>391299</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="16">
         <v>5825</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="18">
         <v>1.49</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="15">
+      <c r="D6" s="16">
         <v>399160</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="16">
         <v>6075</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="18">
         <v>1.52</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D7" s="15">
+        <v>64</v>
+      </c>
+      <c r="D7" s="16">
         <v>406891</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="16">
         <v>6233</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="18">
         <v>1.53</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <v>429444</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="16">
         <v>6536</v>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="18">
         <v>1.52</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="15">
+        <v>64</v>
+      </c>
+      <c r="D9" s="16">
         <v>429291</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="16">
         <v>6190</v>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="18">
         <v>1.44</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D10" s="15">
+        <v>64</v>
+      </c>
+      <c r="D10" s="16">
         <v>429949</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="16">
         <v>6404</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="18">
         <v>1.49</v>
       </c>
     </row>
@@ -1294,13 +1331,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>69</v>
+      <c r="A1" s="22" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.25">
@@ -1311,126 +1348,126 @@
         <v>8</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="15">
-        <v>58</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>75</v>
+        <v>20</v>
+      </c>
+      <c r="C5" s="16">
+        <v>27</v>
+      </c>
+      <c r="D5" s="16">
+        <v>22</v>
+      </c>
+      <c r="E5" s="18">
+        <v>81.48</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="15">
-        <v>47</v>
-      </c>
-      <c r="D6" s="15">
-        <v>43</v>
-      </c>
-      <c r="E6" s="19">
-        <v>91.48999999999999</v>
+        <v>76</v>
+      </c>
+      <c r="C6" s="16">
+        <v>58</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="15">
-        <v>37</v>
-      </c>
-      <c r="D7" s="15">
-        <v>30</v>
-      </c>
-      <c r="E7" s="19">
-        <v>81.08</v>
+        <v>26</v>
+      </c>
+      <c r="C7" s="16">
+        <v>47</v>
+      </c>
+      <c r="D7" s="16">
+        <v>43</v>
+      </c>
+      <c r="E7" s="18">
+        <v>91.48999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="16">
+        <v>31</v>
+      </c>
+      <c r="D8" s="16">
         <v>28</v>
       </c>
-      <c r="C8" s="15">
-        <v>31</v>
-      </c>
-      <c r="D8" s="15">
-        <v>28</v>
-      </c>
-      <c r="E8" s="19">
+      <c r="E8" s="18">
         <v>90.31999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="16">
+        <v>37</v>
+      </c>
+      <c r="D9" s="16">
         <v>30</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="15">
-        <v>27</v>
-      </c>
-      <c r="D9" s="15">
-        <v>22</v>
-      </c>
-      <c r="E9" s="19">
-        <v>81.48</v>
+      <c r="E9" s="18">
+        <v>81.08</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="15">
+        <v>35</v>
+      </c>
+      <c r="C10" s="16">
         <v>26</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <v>23</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="18">
         <v>88.45999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="15">
+        <v>78</v>
+      </c>
+      <c r="C11" s="16">
         <v>19</v>
       </c>
-      <c r="D11" s="22" t="s">
-        <v>75</v>
+      <c r="D11" s="23" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1447,33 +1484,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
+      <c r="A1" s="24" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
+    <row r="2" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+    <row r="3" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+    <row r="4" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="25" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>